<commit_message>
working on handsheet data
</commit_message>
<xml_diff>
--- a/HelloFresh_Absorption.xlsx
+++ b/HelloFresh_Absorption.xlsx
@@ -5,12 +5,12 @@
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://nuwildcat-my.sharepoint.com/personal/stn424_ads_northwestern_edu/Documents/Collaborations/Proposals/GO-Barrier, TFMI Proposals with Tim Wei/URAP_2023-10/Shared/Lanning, Mackenzie/Absorption Data/Fall 2025/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://nuwildcat-my.sharepoint.com/personal/stn424_ads_northwestern_edu/Documents/Collaborations/Proposals/GO-Barrier, TFMI Proposals with Tim Wei/URAP_2023-10/Shared/Lanning, Mackenzie/graphene-oxide-paper-coatings/"/>
     </mc:Choice>
   </mc:AlternateContent>
   <xr:revisionPtr revIDLastSave="2134" documentId="13_ncr:1_{F2E763B4-4DB6-894B-B240-8188D6068E1F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{86EF033D-2D68-2D4E-9CB9-4B2F3C23BAA6}"/>
   <bookViews>
-    <workbookView xWindow="13980" yWindow="740" windowWidth="15420" windowHeight="17180" firstSheet="1" activeTab="5" xr2:uid="{304DC28A-0BB6-064B-B35E-217EA1A1C90F}"/>
+    <workbookView xWindow="13980" yWindow="740" windowWidth="15420" windowHeight="17180" firstSheet="2" activeTab="6" xr2:uid="{304DC28A-0BB6-064B-B35E-217EA1A1C90F}"/>
   </bookViews>
   <sheets>
     <sheet name="Crayola Method" sheetId="1" r:id="rId1"/>
@@ -373,14 +373,14 @@
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="165" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="165" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="49" fontId="2" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="165" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -32320,24 +32320,24 @@
       <c r="P1" s="3"/>
     </row>
     <row r="2" spans="1:18" x14ac:dyDescent="0.2">
-      <c r="A2" s="29" t="s">
-        <v>0</v>
-      </c>
-      <c r="B2" s="29"/>
-      <c r="C2" s="29"/>
-      <c r="D2" s="29"/>
-      <c r="E2" s="29"/>
-      <c r="F2" s="29"/>
-      <c r="G2" s="29"/>
-      <c r="H2" s="29"/>
-      <c r="I2" s="29"/>
-      <c r="J2" s="29"/>
-      <c r="K2" s="29"/>
-      <c r="L2" s="29"/>
-      <c r="M2" s="29"/>
-      <c r="N2" s="29"/>
-      <c r="O2" s="29"/>
-      <c r="P2" s="29"/>
+      <c r="A2" s="30" t="s">
+        <v>0</v>
+      </c>
+      <c r="B2" s="30"/>
+      <c r="C2" s="30"/>
+      <c r="D2" s="30"/>
+      <c r="E2" s="30"/>
+      <c r="F2" s="30"/>
+      <c r="G2" s="30"/>
+      <c r="H2" s="30"/>
+      <c r="I2" s="30"/>
+      <c r="J2" s="30"/>
+      <c r="K2" s="30"/>
+      <c r="L2" s="30"/>
+      <c r="M2" s="30"/>
+      <c r="N2" s="30"/>
+      <c r="O2" s="30"/>
+      <c r="P2" s="30"/>
     </row>
     <row r="3" spans="1:18" ht="51" x14ac:dyDescent="0.2">
       <c r="A3" s="2" t="s">
@@ -34282,24 +34282,24 @@
       <c r="P46" s="5"/>
     </row>
     <row r="47" spans="1:16" x14ac:dyDescent="0.2">
-      <c r="A47" s="30" t="s">
+      <c r="A47" s="31" t="s">
         <v>3</v>
       </c>
-      <c r="B47" s="30"/>
-      <c r="C47" s="30"/>
-      <c r="D47" s="30"/>
-      <c r="E47" s="30"/>
-      <c r="F47" s="30"/>
-      <c r="G47" s="30"/>
-      <c r="H47" s="30"/>
-      <c r="I47" s="30"/>
-      <c r="J47" s="30"/>
-      <c r="K47" s="30"/>
-      <c r="L47" s="30"/>
-      <c r="M47" s="30"/>
-      <c r="N47" s="30"/>
-      <c r="O47" s="30"/>
-      <c r="P47" s="30"/>
+      <c r="B47" s="31"/>
+      <c r="C47" s="31"/>
+      <c r="D47" s="31"/>
+      <c r="E47" s="31"/>
+      <c r="F47" s="31"/>
+      <c r="G47" s="31"/>
+      <c r="H47" s="31"/>
+      <c r="I47" s="31"/>
+      <c r="J47" s="31"/>
+      <c r="K47" s="31"/>
+      <c r="L47" s="31"/>
+      <c r="M47" s="31"/>
+      <c r="N47" s="31"/>
+      <c r="O47" s="31"/>
+      <c r="P47" s="31"/>
     </row>
     <row r="48" spans="1:16" ht="51" x14ac:dyDescent="0.2">
       <c r="A48" s="2" t="s">
@@ -38665,13 +38665,13 @@
       <c r="H1" s="2"/>
     </row>
     <row r="2" spans="1:9" x14ac:dyDescent="0.2">
-      <c r="A2" s="29" t="s">
-        <v>0</v>
-      </c>
-      <c r="B2" s="29"/>
-      <c r="C2" s="29"/>
-      <c r="D2" s="29"/>
-      <c r="E2" s="29"/>
+      <c r="A2" s="30" t="s">
+        <v>0</v>
+      </c>
+      <c r="B2" s="30"/>
+      <c r="C2" s="30"/>
+      <c r="D2" s="30"/>
+      <c r="E2" s="30"/>
       <c r="F2" s="2"/>
       <c r="G2" s="2"/>
       <c r="H2" s="2"/>
@@ -39839,13 +39839,13 @@
       <c r="H52" s="4"/>
     </row>
     <row r="53" spans="1:9" x14ac:dyDescent="0.2">
-      <c r="A53" s="30" t="s">
+      <c r="A53" s="31" t="s">
         <v>3</v>
       </c>
-      <c r="B53" s="30"/>
-      <c r="C53" s="30"/>
-      <c r="D53" s="30"/>
-      <c r="E53" s="30"/>
+      <c r="B53" s="31"/>
+      <c r="C53" s="31"/>
+      <c r="D53" s="31"/>
+      <c r="E53" s="31"/>
       <c r="F53" s="2"/>
       <c r="G53" s="2"/>
       <c r="H53" s="2"/>
@@ -43007,13 +43007,13 @@
       <c r="H1" s="2"/>
     </row>
     <row r="2" spans="1:18" x14ac:dyDescent="0.2">
-      <c r="A2" s="29" t="s">
-        <v>0</v>
-      </c>
-      <c r="B2" s="29"/>
-      <c r="C2" s="29"/>
-      <c r="D2" s="29"/>
-      <c r="E2" s="29"/>
+      <c r="A2" s="30" t="s">
+        <v>0</v>
+      </c>
+      <c r="B2" s="30"/>
+      <c r="C2" s="30"/>
+      <c r="D2" s="30"/>
+      <c r="E2" s="30"/>
       <c r="F2" s="2"/>
       <c r="G2" s="2"/>
       <c r="H2" s="2"/>
@@ -44933,13 +44933,13 @@
       <c r="R52" s="5"/>
     </row>
     <row r="53" spans="1:18" x14ac:dyDescent="0.2">
-      <c r="A53" s="30" t="s">
+      <c r="A53" s="31" t="s">
         <v>3</v>
       </c>
-      <c r="B53" s="30"/>
-      <c r="C53" s="30"/>
-      <c r="D53" s="30"/>
-      <c r="E53" s="30"/>
+      <c r="B53" s="31"/>
+      <c r="C53" s="31"/>
+      <c r="D53" s="31"/>
+      <c r="E53" s="31"/>
       <c r="F53" s="2"/>
       <c r="G53" s="2"/>
       <c r="H53" s="2"/>
@@ -49894,24 +49894,24 @@
       <c r="P1" s="3"/>
     </row>
     <row r="2" spans="1:16" x14ac:dyDescent="0.2">
-      <c r="A2" s="29" t="s">
-        <v>0</v>
-      </c>
-      <c r="B2" s="29"/>
-      <c r="C2" s="29"/>
-      <c r="D2" s="29"/>
-      <c r="E2" s="29"/>
-      <c r="F2" s="29"/>
-      <c r="G2" s="29"/>
-      <c r="H2" s="29"/>
-      <c r="I2" s="29"/>
-      <c r="J2" s="29"/>
-      <c r="K2" s="29"/>
-      <c r="L2" s="29"/>
-      <c r="M2" s="29"/>
-      <c r="N2" s="29"/>
-      <c r="O2" s="29"/>
-      <c r="P2" s="29"/>
+      <c r="A2" s="30" t="s">
+        <v>0</v>
+      </c>
+      <c r="B2" s="30"/>
+      <c r="C2" s="30"/>
+      <c r="D2" s="30"/>
+      <c r="E2" s="30"/>
+      <c r="F2" s="30"/>
+      <c r="G2" s="30"/>
+      <c r="H2" s="30"/>
+      <c r="I2" s="30"/>
+      <c r="J2" s="30"/>
+      <c r="K2" s="30"/>
+      <c r="L2" s="30"/>
+      <c r="M2" s="30"/>
+      <c r="N2" s="30"/>
+      <c r="O2" s="30"/>
+      <c r="P2" s="30"/>
     </row>
     <row r="3" spans="1:16" ht="34" x14ac:dyDescent="0.2">
       <c r="A3" s="2" t="s">
@@ -51138,24 +51138,24 @@
       <c r="P46" s="5"/>
     </row>
     <row r="47" spans="1:16" x14ac:dyDescent="0.2">
-      <c r="A47" s="30" t="s">
+      <c r="A47" s="31" t="s">
         <v>3</v>
       </c>
-      <c r="B47" s="30"/>
-      <c r="C47" s="30"/>
-      <c r="D47" s="30"/>
-      <c r="E47" s="30"/>
-      <c r="F47" s="30"/>
-      <c r="G47" s="30"/>
-      <c r="H47" s="30"/>
-      <c r="I47" s="30"/>
-      <c r="J47" s="30"/>
-      <c r="K47" s="30"/>
-      <c r="L47" s="30"/>
-      <c r="M47" s="30"/>
-      <c r="N47" s="30"/>
-      <c r="O47" s="30"/>
-      <c r="P47" s="30"/>
+      <c r="B47" s="31"/>
+      <c r="C47" s="31"/>
+      <c r="D47" s="31"/>
+      <c r="E47" s="31"/>
+      <c r="F47" s="31"/>
+      <c r="G47" s="31"/>
+      <c r="H47" s="31"/>
+      <c r="I47" s="31"/>
+      <c r="J47" s="31"/>
+      <c r="K47" s="31"/>
+      <c r="L47" s="31"/>
+      <c r="M47" s="31"/>
+      <c r="N47" s="31"/>
+      <c r="O47" s="31"/>
+      <c r="P47" s="31"/>
     </row>
     <row r="48" spans="1:16" ht="34" x14ac:dyDescent="0.2">
       <c r="A48" s="2" t="s">
@@ -59979,7 +59979,7 @@
       <c r="C1" s="25" t="s">
         <v>50</v>
       </c>
-      <c r="D1" s="31" t="s">
+      <c r="D1" s="29" t="s">
         <v>58</v>
       </c>
     </row>

</xml_diff>